<commit_message>
Document Python version, soften licensing wording, remove scratch columns from panels
</commit_message>
<xml_diff>
--- a/data/mastersheet_epu.xlsx
+++ b/data/mastersheet_epu.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2932"/>
+  <dimension ref="A1:K2932"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -596,11 +596,6 @@
       <c r="I3" t="n">
         <v>370.174951165918</v>
       </c>
-      <c r="N3" s="9" t="inlineStr">
-        <is>
-          <t>Counts</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -632,26 +627,6 @@
       <c r="I4" t="n">
         <v>422.187035160094</v>
       </c>
-      <c r="N4" s="1" t="inlineStr">
-        <is>
-          <t>Announcement</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>Stress</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>Non stress</t>
-        </is>
-      </c>
-      <c r="Q4" s="1" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -683,18 +658,6 @@
       <c r="I5" t="n">
         <v>422.187035160094</v>
       </c>
-      <c r="N5" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -726,18 +689,6 @@
       <c r="I6" t="n">
         <v>424.123448713137</v>
       </c>
-      <c r="N6" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -769,18 +720,6 @@
       <c r="I7" t="n">
         <v>424.123448713137</v>
       </c>
-      <c r="N7" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -812,18 +751,6 @@
       <c r="I8" t="n">
         <v>396.778288530327</v>
       </c>
-      <c r="N8" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -855,18 +782,6 @@
       <c r="I9" t="n">
         <v>375.563447990337</v>
       </c>
-      <c r="N9" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -898,18 +813,6 @@
       <c r="I10" t="n">
         <v>322.081266386477</v>
       </c>
-      <c r="N10" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -941,18 +844,6 @@
       <c r="I11" t="n">
         <v>447.404458770102</v>
       </c>
-      <c r="N11" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -984,18 +875,6 @@
       <c r="I12" t="n">
         <v>494.283888682785</v>
       </c>
-      <c r="N12" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1027,18 +906,6 @@
       <c r="I13" t="n">
         <v>618.6626574377329</v>
       </c>
-      <c r="N13" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1070,18 +937,6 @@
       <c r="I14" t="n">
         <v>688.948013134432</v>
       </c>
-      <c r="N14" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1113,18 +968,6 @@
       <c r="I15" t="n">
         <v>625.94934353999</v>
       </c>
-      <c r="N15" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1156,18 +999,6 @@
       <c r="I16" t="n">
         <v>366.303412813377</v>
       </c>
-      <c r="N16" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1199,18 +1030,6 @@
       <c r="I17" t="n">
         <v>291.740459718168</v>
       </c>
-      <c r="N17" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1242,18 +1061,6 @@
       <c r="I18" t="n">
         <v>182.712970715509</v>
       </c>
-      <c r="N18" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1284,18 +1091,6 @@
       </c>
       <c r="I19" t="n">
         <v>236.745896877256</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0.4166666666666666</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="20">

</xml_diff>